<commit_message>
velky update a event skill
</commit_message>
<xml_diff>
--- a/skills/xlab-pricing/data/XLAB_Centralni_Cenik_v5.xlsx
+++ b/skills/xlab-pricing/data/XLAB_Centralni_Cenik_v5.xlsx
@@ -254,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -348,6 +348,7 @@
     <xf numFmtId="3" fontId="16" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="17" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -713,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1475,16 +1476,16 @@
         </is>
       </c>
       <c r="D28" s="47" t="n">
+        <v>650</v>
+      </c>
+      <c r="E28" s="34" t="n">
+        <v>750</v>
+      </c>
+      <c r="F28" s="34" t="n">
         <v>900</v>
       </c>
-      <c r="E28" s="34" t="n">
-        <v>900</v>
-      </c>
-      <c r="F28" s="34" t="n">
+      <c r="G28" s="34" t="n">
         <v>1100</v>
-      </c>
-      <c r="G28" s="34" t="n">
-        <v>1300</v>
       </c>
       <c r="H28" s="36" t="n"/>
       <c r="I28" s="48" t="n">
@@ -1494,7 +1495,12 @@
     <row r="29">
       <c r="A29" s="33" t="inlineStr">
         <is>
-          <t>Video Operator</t>
+          <t>Sound Operator</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Obsluha zvukové techniky, mix, mikrofony</t>
         </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
@@ -1503,30 +1509,23 @@
         </is>
       </c>
       <c r="D29" s="47" t="n">
+        <v>650</v>
+      </c>
+      <c r="E29" s="34" t="n">
         <v>750</v>
       </c>
-      <c r="E29" s="34" t="n">
+      <c r="F29" s="34" t="n">
         <v>900</v>
       </c>
-      <c r="F29" s="34" t="n">
+      <c r="G29" s="34" t="n">
         <v>1100</v>
       </c>
-      <c r="G29" s="34" t="n">
-        <v>1300</v>
-      </c>
-      <c r="H29" s="38" t="inlineStr">
-        <is>
-          <t>Pro setupy bez 3D Media Serveru</t>
-        </is>
-      </c>
-      <c r="I29" s="48" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H29" s="36" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="33" t="inlineStr">
         <is>
-          <t>3D Media Server Operator</t>
+          <t>Video Operator</t>
         </is>
       </c>
       <c r="C30" s="33" t="inlineStr">
@@ -1535,100 +1534,104 @@
         </is>
       </c>
       <c r="D30" s="47" t="n">
-        <v>1000</v>
+        <v>650</v>
       </c>
       <c r="E30" s="34" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="F30" s="34" t="n">
-        <v>1250</v>
+        <v>950</v>
       </c>
       <c r="G30" s="34" t="n">
-        <v>1500</v>
+        <v>1150</v>
       </c>
       <c r="H30" s="38" t="inlineStr">
         <is>
-          <t>3D Server setup — vyžaduje specializaci</t>
+          <t>Pro setupy bez 3D Media Serveru</t>
         </is>
       </c>
       <c r="I30" s="48" t="n">
-        <v>14000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="33" t="inlineStr">
         <is>
+          <t>3D Media Server Operator</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
+          <t>CZK/h</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E31" s="34" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F31" s="34" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G31" s="34" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H31" s="38" t="inlineStr">
+        <is>
+          <t>3D Server setup — vyžaduje specializaci</t>
+        </is>
+      </c>
+      <c r="I31" s="48" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="33" t="inlineStr">
+        <is>
           <t>Technical Engineer</t>
         </is>
       </c>
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C32" s="33" t="inlineStr">
         <is>
           <t>CZK/h</t>
         </is>
       </c>
-      <c r="D31" s="47" t="n">
+      <c r="D32" s="47" t="n">
         <v>550</v>
       </c>
-      <c r="E31" s="34" t="n">
+      <c r="E32" s="34" t="n">
         <v>750</v>
       </c>
-      <c r="F31" s="34" t="n">
+      <c r="F32" s="34" t="n">
         <v>950</v>
       </c>
-      <c r="G31" s="34" t="n">
+      <c r="G32" s="34" t="n">
         <v>1150</v>
       </c>
-      <c r="H31" s="36" t="n"/>
-      <c r="I31" s="48" t="n">
+      <c r="H32" s="36" t="n"/>
+      <c r="I32" s="48" t="n">
         <v>9000</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="31" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t>AI &amp; AVATAR DEVELOPMENT</t>
         </is>
       </c>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="32" t="n"/>
-      <c r="E32" s="32" t="n"/>
-      <c r="F32" s="32" t="n"/>
-      <c r="G32" s="32" t="n"/>
-      <c r="H32" s="32" t="n"/>
-      <c r="I32" s="36" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="33" t="inlineStr">
-        <is>
-          <t>Brain Development and Setup</t>
-        </is>
-      </c>
-      <c r="C33" s="33" t="inlineStr">
-        <is>
-          <t>CZK/h</t>
-        </is>
-      </c>
-      <c r="D33" s="47" t="n">
-        <v>500</v>
-      </c>
-      <c r="E33" s="34" t="n">
-        <v>950</v>
-      </c>
-      <c r="F33" s="34" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G33" s="34" t="n">
-        <v>1450</v>
-      </c>
-      <c r="H33" s="36" t="n"/>
-      <c r="I33" s="48" t="n">
-        <v>11000</v>
-      </c>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="32" t="n"/>
+      <c r="F33" s="32" t="n"/>
+      <c r="G33" s="32" t="n"/>
+      <c r="H33" s="32" t="n"/>
+      <c r="I33" s="36" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="33" t="inlineStr">
         <is>
-          <t>Brain Customization and Testing</t>
+          <t>Brain Development and Setup</t>
         </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
@@ -1656,7 +1659,7 @@
     <row r="35">
       <c r="A35" s="33" t="inlineStr">
         <is>
-          <t>Clients Data</t>
+          <t>Brain Customization and Testing</t>
         </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
@@ -1684,7 +1687,7 @@
     <row r="36">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>Personality Setup</t>
+          <t>Clients Data</t>
         </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
@@ -1712,7 +1715,7 @@
     <row r="37">
       <c r="A37" s="33" t="inlineStr">
         <is>
-          <t>Script &amp; Copy</t>
+          <t>Personality Setup</t>
         </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
@@ -1740,7 +1743,7 @@
     <row r="38">
       <c r="A38" s="33" t="inlineStr">
         <is>
-          <t>3D Content Creation</t>
+          <t>Script &amp; Copy</t>
         </is>
       </c>
       <c r="C38" s="33" t="inlineStr">
@@ -1749,68 +1752,68 @@
         </is>
       </c>
       <c r="D38" s="47" t="n">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="E38" s="34" t="n">
+        <v>950</v>
+      </c>
+      <c r="F38" s="34" t="n">
         <v>1200</v>
       </c>
-      <c r="F38" s="34" t="n">
-        <v>1500</v>
-      </c>
       <c r="G38" s="34" t="n">
-        <v>1800</v>
+        <v>1450</v>
       </c>
       <c r="H38" s="36" t="n"/>
       <c r="I38" s="48" t="n">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="33" t="inlineStr">
+        <is>
+          <t>3D Content Creation</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>CZK/h</t>
+        </is>
+      </c>
+      <c r="D39" s="47" t="n">
+        <v>900</v>
+      </c>
+      <c r="E39" s="34" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F39" s="34" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G39" s="34" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H39" s="36" t="n"/>
+      <c r="I39" s="48" t="n">
         <v>14000</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="31" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="31" t="inlineStr">
         <is>
           <t>ON-SITE PRODUKCE</t>
         </is>
       </c>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="32" t="n"/>
-      <c r="F39" s="32" t="n"/>
-      <c r="G39" s="32" t="n"/>
-      <c r="H39" s="32" t="n"/>
-      <c r="I39" s="36" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="33" t="inlineStr">
-        <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="C40" s="33" t="inlineStr">
-        <is>
-          <t>CZK/h</t>
-        </is>
-      </c>
-      <c r="D40" s="47" t="n">
-        <v>550</v>
-      </c>
-      <c r="E40" s="34" t="n">
-        <v>900</v>
-      </c>
-      <c r="F40" s="34" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G40" s="34" t="n">
-        <v>1300</v>
-      </c>
-      <c r="H40" s="36" t="n"/>
-      <c r="I40" s="48" t="n">
-        <v>10000</v>
-      </c>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="32" t="n"/>
+      <c r="E40" s="32" t="n"/>
+      <c r="F40" s="32" t="n"/>
+      <c r="G40" s="32" t="n"/>
+      <c r="H40" s="32" t="n"/>
+      <c r="I40" s="36" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="33" t="inlineStr">
         <is>
-          <t>Showcall / Director</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="C41" s="33" t="inlineStr">
@@ -1819,26 +1822,26 @@
         </is>
       </c>
       <c r="D41" s="47" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="E41" s="34" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="F41" s="34" t="n">
-        <v>1250</v>
+        <v>1100</v>
       </c>
       <c r="G41" s="34" t="n">
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="H41" s="36" t="n"/>
       <c r="I41" s="48" t="n">
-        <v>11000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="33" t="inlineStr">
         <is>
-          <t>DJ Operator / Sound Designer vč. techniky</t>
+          <t>Showcall / Director</t>
         </is>
       </c>
       <c r="C42" s="33" t="inlineStr">
@@ -1847,7 +1850,7 @@
         </is>
       </c>
       <c r="D42" s="47" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="E42" s="34" t="n">
         <v>1000</v>
@@ -1866,7 +1869,7 @@
     <row r="43">
       <c r="A43" s="33" t="inlineStr">
         <is>
-          <t>Stage Hands</t>
+          <t>DJ Operator / Sound Designer vč. techniky</t>
         </is>
       </c>
       <c r="C43" s="33" t="inlineStr">
@@ -1875,55 +1878,83 @@
         </is>
       </c>
       <c r="D43" s="47" t="n">
-        <v>450</v>
+        <v>750</v>
       </c>
       <c r="E43" s="34" t="n">
-        <v>550</v>
+        <v>1000</v>
       </c>
       <c r="F43" s="34" t="n">
-        <v>550</v>
+        <v>1250</v>
       </c>
       <c r="G43" s="34" t="n">
-        <v>650</v>
-      </c>
-      <c r="H43" s="38" t="inlineStr">
-        <is>
-          <t>Snížená = Standard</t>
-        </is>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="H43" s="36" t="n"/>
       <c r="I43" s="48" t="n">
-        <v>5000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="33" t="inlineStr">
         <is>
+          <t>Stage Hands</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>CZK/h</t>
+        </is>
+      </c>
+      <c r="D44" s="47" t="n">
+        <v>450</v>
+      </c>
+      <c r="E44" s="34" t="n">
+        <v>550</v>
+      </c>
+      <c r="F44" s="34" t="n">
+        <v>550</v>
+      </c>
+      <c r="G44" s="34" t="n">
+        <v>650</v>
+      </c>
+      <c r="H44" s="38" t="inlineStr">
+        <is>
+          <t>Snížená = Standard</t>
+        </is>
+      </c>
+      <c r="I44" s="48" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="inlineStr">
+        <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C44" s="33" t="inlineStr">
+      <c r="C45" s="33" t="inlineStr">
         <is>
           <t>CZK/den</t>
         </is>
       </c>
-      <c r="D44" s="47" t="n">
+      <c r="D45" s="47" t="n">
         <v>5200</v>
       </c>
-      <c r="E44" s="34" t="n">
+      <c r="E45" s="34" t="n">
         <v>6400</v>
       </c>
-      <c r="F44" s="34" t="n">
+      <c r="F45" s="34" t="n">
         <v>8000</v>
       </c>
-      <c r="G44" s="34" t="n">
+      <c r="G45" s="34" t="n">
         <v>9600</v>
       </c>
-      <c r="H44" s="38" t="inlineStr">
+      <c r="H45" s="38" t="inlineStr">
         <is>
           <t>Paušál/den</t>
         </is>
       </c>
-      <c r="I44" s="48" t="n">
+      <c r="I45" s="48" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -1938,7 +1969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2785,7 +2816,7 @@
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t>AI AVATAR &amp; HOLOBOX HARDWARE</t>
+          <t>AI AVATAR &amp; HOLOBOX</t>
         </is>
       </c>
       <c r="C35" s="32" t="n"/>
@@ -2798,7 +2829,12 @@
     <row r="36">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>AI Avatar Hardware — rental</t>
+          <t>Holobox — pronájem jednotky</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pronájem Holobox displeje (životní velikost, 4K) vč. dopravy a instalace</t>
         </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
@@ -2810,15 +2846,321 @@
         <v>3000</v>
       </c>
       <c r="E36" s="34" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F36" s="34" t="n">
         <v>20000</v>
       </c>
-      <c r="F36" s="34" t="n">
-        <v>25000</v>
-      </c>
       <c r="G36" s="34" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H36" s="36" t="n"/>
+        <v>24000</v>
+      </c>
+      <c r="H36" s="36" t="inlineStr">
+        <is>
+          <t>Hardware — fyzická jednotka</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="33" t="inlineStr">
+        <is>
+          <t>AI Avatar — licence a nastavení</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Digitální osoba: vzhled, hlas, základní brain</t>
+        </is>
+      </c>
+      <c r="C37" s="33" t="inlineStr">
+        <is>
+          <t>CZK/set/den</t>
+        </is>
+      </c>
+      <c r="D37" s="49" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E37" s="33" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F37" s="33" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G37" s="33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H37" s="36" t="inlineStr">
+        <is>
+          <t>SW licence — bez brain development</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>OSVĚTLENÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LED PAR 100W</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plošné / akcentní nasvícení (cena za kus)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CZK/ks/den</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>300</v>
+      </c>
+      <c r="E40" t="n">
+        <v>450</v>
+      </c>
+      <c r="F40" t="n">
+        <v>550</v>
+      </c>
+      <c r="G40" t="n">
+        <v>650</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Ambient i akcent</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Profilový reflektor</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Směrové nasvícení objektů, osob, scény</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CZK/ks/den</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>500</v>
+      </c>
+      <c r="E41" t="n">
+        <v>700</v>
+      </c>
+      <c r="F41" t="n">
+        <v>900</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Světelný pult + show control</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Řídící pult světel vč. programování cues</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CZK/set/den</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>900</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ZVUK</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PA systém — ozvučení sálu</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Reproboxy + zesilovač, pokrytí středního sálu</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CZK/set/den</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E45" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F45" t="n">
+        <v>17500</v>
+      </c>
+      <c r="G45" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Rozsah dle velikosti sálu</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mixážní pult</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Digitální mixpult vč. kabeláže</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CZK/set/den</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>900</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Mikrofonní stojka</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Statický mikrofon na pódiu vč. stojanu</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CZK/ks/den</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>500</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Bezdrátový mikrofon — handka</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ruční bezdrátový mikrofon</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CZK/ks/den</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>KABELÁŽ &amp; INFRASTRUKTURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Kabeláž + spojovací materiál</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Silové + signálové kabely, konektory, instalace</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CZK/set</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F51" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G51" t="n">
+        <v>6000</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Dle rozsahu akce — 4k–6k snížená</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4412,7 +4754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J191"/>
+  <dimension ref="A1:J236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8457,7 +8799,7 @@
       </c>
       <c r="B151" s="33" t="inlineStr">
         <is>
-          <t>AI Avatar HW — rental</t>
+          <t>Holobox — pronájem jednotky</t>
         </is>
       </c>
       <c r="C151" s="33" t="inlineStr">
@@ -8475,17 +8817,17 @@
         <v>1.5</v>
       </c>
       <c r="G151" s="34" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="H151" s="34" t="n">
-        <v>37500</v>
+        <v>30000</v>
       </c>
       <c r="I151" s="34" t="n">
-        <v>37500</v>
+        <v>30000</v>
       </c>
       <c r="J151" s="38" t="inlineStr">
         <is>
-          <t>25 000/set/den</t>
+          <t>20 000/set/den</t>
         </is>
       </c>
     </row>
@@ -8647,22 +8989,22 @@
         </is>
       </c>
       <c r="D157" s="33" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E157" s="33" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F157" s="33" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G157" s="34" t="n">
-        <v>4400</v>
+        <v>8800</v>
       </c>
       <c r="H157" s="34" t="n">
-        <v>6600</v>
+        <v>13200</v>
       </c>
       <c r="I157" s="34" t="n">
-        <v>8800</v>
+        <v>17600</v>
       </c>
       <c r="J157" s="38" t="inlineStr">
         <is>
@@ -8893,13 +9235,13 @@
       <c r="E165" s="44" t="n"/>
       <c r="F165" s="44" t="n"/>
       <c r="G165" s="46" t="n">
-        <v>64450</v>
+        <v>63850</v>
       </c>
       <c r="H165" s="46" t="n">
-        <v>108450</v>
+        <v>107550</v>
       </c>
       <c r="I165" s="46" t="n">
-        <v>174900</v>
+        <v>176200</v>
       </c>
       <c r="J165" s="44" t="n"/>
     </row>
@@ -9621,6 +9963,993 @@
         <v>927100</v>
       </c>
       <c r="J191" s="44" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>MENŠÍ EVENT — OZVUČENÍ &amp; NASVÍCENÍ (Vernisáž)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Lidé — příprava</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>1</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>3</v>
+      </c>
+      <c r="E195" t="n">
+        <v>4</v>
+      </c>
+      <c r="F195" t="n">
+        <v>6</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Řízení projektu</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>2</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Technical Production</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>3</v>
+      </c>
+      <c r="E196" t="n">
+        <v>4</v>
+      </c>
+      <c r="F196" t="n">
+        <v>6</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Technická příprava</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Lidé — na místě</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>3</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>3</v>
+      </c>
+      <c r="E198" t="n">
+        <v>10</v>
+      </c>
+      <c r="F198" t="n">
+        <v>10</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>900/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>4</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Light Designer</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>8</v>
+      </c>
+      <c r="E199" t="n">
+        <v>10</v>
+      </c>
+      <c r="F199" t="n">
+        <v>12</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>900/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>5</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Sound Operator</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>8</v>
+      </c>
+      <c r="E200" t="n">
+        <v>10</v>
+      </c>
+      <c r="F200" t="n">
+        <v>12</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>900/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>6</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Stage Hands</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>os×h</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>12</v>
+      </c>
+      <c r="E201" t="n">
+        <v>20</v>
+      </c>
+      <c r="F201" t="n">
+        <v>24</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>550/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>7</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Technical Engineer</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>8</v>
+      </c>
+      <c r="E202" t="n">
+        <v>10</v>
+      </c>
+      <c r="F202" t="n">
+        <v>12</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>950/h zvukař</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Technika</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>8</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>LED PAR 100W — ambient</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>ks/den</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>12</v>
+      </c>
+      <c r="E204" t="n">
+        <v>24</v>
+      </c>
+      <c r="F204" t="n">
+        <v>30</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>550/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>9</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>LED PAR 100W — akcent</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ks/den</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" t="n">
+        <v>6</v>
+      </c>
+      <c r="F205" t="n">
+        <v>8</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>550/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>10</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Profilový reflektor</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ks/den</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" t="n">
+        <v>2</v>
+      </c>
+      <c r="F206" t="n">
+        <v>4</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>900/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>11</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Světelný pult + show control</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>set/den</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>1</v>
+      </c>
+      <c r="E207" t="n">
+        <v>1</v>
+      </c>
+      <c r="F207" t="n">
+        <v>1</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>1 900/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>12</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>PA systém — ozvučení sálu</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>set/den</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" t="n">
+        <v>1</v>
+      </c>
+      <c r="F208" t="n">
+        <v>1</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>17 500/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>13</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Mixážní pult</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>set/den</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>1</v>
+      </c>
+      <c r="E209" t="n">
+        <v>1</v>
+      </c>
+      <c r="F209" t="n">
+        <v>1</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>1 900/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>14</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Mikrofonní stojka</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ks/den</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>0</v>
+      </c>
+      <c r="E210" t="n">
+        <v>1</v>
+      </c>
+      <c r="F210" t="n">
+        <v>2</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>1 300/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>15</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Bezdrátový mikrofon — handka</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>ks/den</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>0</v>
+      </c>
+      <c r="E211" t="n">
+        <v>1</v>
+      </c>
+      <c r="F211" t="n">
+        <v>2</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>2 250/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>16</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Kabeláž + spojovací materiál</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>1</v>
+      </c>
+      <c r="E212" t="n">
+        <v>1</v>
+      </c>
+      <c r="F212" t="n">
+        <v>1</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>5 000/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Logistika</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>17</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Van — equipment</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>trip</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
+      </c>
+      <c r="E214" t="n">
+        <v>1</v>
+      </c>
+      <c r="F214" t="n">
+        <v>2</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>2 500/trip</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Video add-on (volitelné)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>18</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>LED screen 3×2,5 m</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>set/den</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>0</v>
+      </c>
+      <c r="E216" t="n">
+        <v>1</v>
+      </c>
+      <c r="F216" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>20 000/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>19</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>PPT Setup</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>0</v>
+      </c>
+      <c r="E217" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" t="n">
+        <v>1</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>9 000/set</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>20</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Video Operator</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>0</v>
+      </c>
+      <c r="E218" t="n">
+        <v>10</v>
+      </c>
+      <c r="F218" t="n">
+        <v>10</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>950/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>CELKEM (bez videa)</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H220" t="n">
+        <v>75000</v>
+      </c>
+      <c r="I220" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>CELKEM (s malým videem)</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H221" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I221" t="n">
+        <v>155000</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>AI AVATAR RENTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Koordinace</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>1</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Technical Production</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>4</v>
+      </c>
+      <c r="E225" t="n">
+        <v>6</v>
+      </c>
+      <c r="F225" t="n">
+        <v>8</v>
+      </c>
+      <c r="G225" t="n">
+        <v>4800</v>
+      </c>
+      <c r="H225" t="n">
+        <v>7200</v>
+      </c>
+      <c r="I225" t="n">
+        <v>9600</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>1 200/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>2</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>3</v>
+      </c>
+      <c r="E226" t="n">
+        <v>4</v>
+      </c>
+      <c r="F226" t="n">
+        <v>6</v>
+      </c>
+      <c r="G226" t="n">
+        <v>3750</v>
+      </c>
+      <c r="H226" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I226" t="n">
+        <v>7500</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>1 250/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Technika</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>3</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>AI Avatar — pronájem</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>set/den</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>1</v>
+      </c>
+      <c r="E228" t="n">
+        <v>1</v>
+      </c>
+      <c r="F228" t="n">
+        <v>1</v>
+      </c>
+      <c r="G228" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H228" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I228" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>10 000/set/den</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>AI Avatar — nastavení</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>4</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>AI Avatar — licence a nastavení</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>4</v>
+      </c>
+      <c r="E230" t="n">
+        <v>8</v>
+      </c>
+      <c r="F230" t="n">
+        <v>12</v>
+      </c>
+      <c r="G230" t="n">
+        <v>4800</v>
+      </c>
+      <c r="H230" t="n">
+        <v>9600</v>
+      </c>
+      <c r="I230" t="n">
+        <v>14400</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>1 200/h — brain, vzhled, hlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>5</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Technical support ON SITE</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>os×h</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>8</v>
+      </c>
+      <c r="E232" t="n">
+        <v>9</v>
+      </c>
+      <c r="F232" t="n">
+        <v>10</v>
+      </c>
+      <c r="G232" t="n">
+        <v>7600</v>
+      </c>
+      <c r="H232" t="n">
+        <v>8550</v>
+      </c>
+      <c r="I232" t="n">
+        <v>9500</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>950/h — 1 osoba</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>6</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Load IN / OUT (Stage Hands)</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>os×h</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>12</v>
+      </c>
+      <c r="E233" t="n">
+        <v>16</v>
+      </c>
+      <c r="F233" t="n">
+        <v>18</v>
+      </c>
+      <c r="G233" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H233" t="n">
+        <v>8800</v>
+      </c>
+      <c r="I233" t="n">
+        <v>9900</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>550/h — 2 osoby</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>7</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>trip</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E234" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" t="n">
+        <v>2</v>
+      </c>
+      <c r="G234" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H234" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I234" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Agency fee</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>5,5 %</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H235" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I235" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>CELKEM</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>42050</v>
+      </c>
+      <c r="H236" t="n">
+        <v>54650</v>
+      </c>
+      <c r="I236" t="n">
+        <v>69900</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="43">
@@ -9678,7 +11007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9994,12 +11323,12 @@
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>50–100 tis.</t>
+          <t>40–70 tis.</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>PM + Brain + HW rental (25k) + Tech support + Transport</t>
+          <t>PM + TechProd + Avatar pronájem (10k) + Brain setup + Tech support + Stage Hands (2 os) + Transport</t>
         </is>
       </c>
       <c r="D18" s="38" t="inlineStr">
@@ -10078,6 +11407,57 @@
       <c r="D22" s="38" t="inlineStr">
         <is>
           <t>Bobcat = 645k</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MENŠÍ EVENTY — OZVUČENÍ &amp; NASVÍCENÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Vernisáž / menší event (bez videa)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>50–80 tis.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PM + Light Designer + Sound Op + Stage Hands + PA + LED PAR + Pult + Transport</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NM Palacký</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Vernisáž / menší event (s malým videem)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>100–150 tis.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PM + Light + Sound + Video Op + Stage Hands + PA + LED PAR + Pult + LED screen 3×2,5 + PPT Setup + Pódium + Transport</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NM Přemyslovci</t>
         </is>
       </c>
     </row>

</xml_diff>